<commit_message>
feat(F-NAR-019): ATOM-COL.POL.001-09 Le fromage de Nina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.POL.001-09.xlsx
+++ b/stories/arbres/ATOM-COL.POL.001-09.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le morceau frais de Nina</t>
+          <t>Le fromage de Nina</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>fromagerie, linge blanc, cloche de verre</t>
+          <t>fromagerie, linge blanc à trous, cloche de verre, marbre froid, lait, morceau beige</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut le petit morceau beige sous le linge à trous. Elle dit bonjour, s'il te plaît, merci. Le sac reste froid.</t>
+          <t>Le verre de la cloche est froid. Sur le verre, un éclat de cloche luit. Nina veut le morceau beige maintenant. Elle tend la main trop vite, sans le mot : le verre arrête le doigt. La dame ne lève pas les yeux. Elle refuse de foncer, dit bonjour, obtient le sac. Merci vécu. Elle soulève trop vite : la cloche glisse. Un éclat de cloche reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un linge blanc a de petits trous. Un rayon y passe, tout pâle. Ça sent le lait froid. Des fromages ronds dorment dessous. Une cloche de verre tient un morceau. Le verre est un peu embué, tout doux. Tu as vu les trous, Nina ? Comme des fenêtres. Tout petits. Papa pousse la porte tout doux. Un souffle frais sort de la boutique. Une petite cloche fait ding, tout bas. Tu as senti le lait, Nina ? Oui, maman. C'est frais. Comme le matin. Le carrelage est froid sous les chaussures. Tu as les pieds froids, Nina ? Un peu, maman. En ce moment, Nina s'arrête au comptoir. Un petit morceau beige est sur une feuille. La feuille craque un peu. Celui-là, papa. On s'approche du comptoir. Elle plie encore le linge. Nina se tient près de maman. Elle regarde par un trou du linge. Je vois le morceau. Oui. La dame pose le linge. Elle lève les yeux. Tu demandes, Nina.</t>
+          <t>Le verre de la cloche est froid. Un rayon pâle y glisse. Sur le verre, un éclat de cloche luit. Il brille, papa. Tu le vois, sur le verre ? Nina pose un doigt, un instant. Le verre pique un peu le doigt. Il est froid. La veste, un bouton de plus. Voilà. Un souffle frais sort de la boutique. J'ai les joues froides. On avance. Tu restes près de nous ? Oui, maman. Ça sent le lait, près du verre. Des ronds dorment sous le linge. Ça sent le lait ! Tu sens, Nina ? Oui. Le linge blanc a de petits trous. Le carrelage est froid sous les chaussures. On reste près du marbre. Le marbre du comptoir est lisse. Le linge sent le lait, un peu. Nina regarde par un trou du linge. Je vois le morceau. Par un trou, Nina ? Oui, maman. Je le veux, maintenant. En ce moment, Nina serre la veste. Le sol est froid sous ses chaussures. Une feuille craque sous un morceau. Celui-là ! Nina se dresse sur les pointes. Un petit morceau beige attend sous le verre. Nina tend la main trop vite. Je le prends ! Le doigt tape le verre. Oh. Le morceau reste sous la cloche. La dame ne lève pas les yeux. Le sourire de Nina disparaît. Il ne vient pas. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Le fromage est sous le verre. Tu le vois, Nina ? Les épaules de Nina tombent un peu. Ça serre, dans son ventre. L'éclat de cloche tremble, puis tient. Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un linge blanc a de petits trous. Un rayon y passe, tout pâle. Ça sent le lait froid. Des fromages ronds dorment dessous. Une cloche de verre tient un morceau. Le verre est un peu embué, tout doux. Tu as vu les trous, Nina ? Comme des fenêtres. Tout petits. Papa pousse la porte tout doux. Un souffle frais sort de la boutique. Une petite cloche fait ding, tout bas. Tu as senti le lait, Nina ? Oui, maman. C'est frais. Comme le matin. Le carrelage est froid sous les chaussures. Tu as les pieds froids, Nina ? Un peu, maman. En ce moment, Nina s'arrête au comptoir. Un petit morceau beige est sur une feuille. La feuille craque un peu. Celui-là, papa. On s'approche du comptoir. Elle plie encore le linge. Nina se tient près de maman. Elle regarde par un trou du linge. Je vois le morceau. Oui. La dame pose le linge. Elle lève les yeux. Tu demandes, Nina.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le verre de la cloche est froid. Un rayon pâle y glisse. Sur le verre, un &lt;emphasis level="moderate"&gt;éclat de cloche&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur le verre ? Nina pose un doigt, un instant. Le verre pique un peu le doigt. Il est froid. La veste, un bouton de plus. Voilà. Un souffle frais sort de la boutique. J'ai les joues froides. On avance. Tu restes près de nous ? Oui, maman. Ça sent le lait, près du verre. Des ronds dorment sous le linge. Ça sent le lait ! Tu sens, Nina ? Oui. Le linge blanc a de petits trous. Le carrelage est froid sous les chaussures. On reste près du marbre. Le marbre du comptoir est lisse. Le linge sent le lait, un peu. Nina regarde par un trou du linge. Je vois le morceau. Par un trou, Nina ? Oui, maman. Je le veux, maintenant. En ce moment, Nina serre la veste. Le sol est froid sous ses chaussures. Une feuille craque sous un morceau. Celui-là ! Nina se dresse sur les pointes. Un petit morceau beige attend sous le verre. Nina tend la main trop vite. Je le prends ! Le doigt tape le verre. Oh. Le morceau reste sous la cloche. La dame ne lève pas les yeux. Le sourire de Nina disparaît. Il ne vient pas. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Le fromage est sous le verre. Tu le vois, Nina ? Les épaules de Nina tombent un peu. Ça serre, dans son ventre. L'éclat de cloche tremble, puis tient. Papa se baisse à sa hauteur.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;David entre à la fromagerie. Papa tient sa main. David dit : &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. L'odeur du fromage est douce. David pointe un morceau. Il dit : s'il te plaît. La dame tend le sac. David dit : merci. Papa sourit. Ils sortent. Le sac est frais. David répète : bonjour. S'il te plaît. Merci. Maman les attend. David dit : merci, maman. Maman dit : bonjour, David. Ils rentrent.&lt;/slow&gt; [pause]</t>
+          <t>Le verre de la cloche est froid. Un rayon pâle y glisse. Sur le verre, un &lt;emphasis&gt;éclat de cloche&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur le verre ? Nina pose un doigt, un instant. Le verre pique un peu le doigt. Il est froid. La veste, un bouton de plus. Voilà. Un souffle frais sort de la boutique. J'ai les joues froides. On avance. Tu restes près de nous ? Oui, maman. Ça sent le lait, près du verre. Des ronds dorment sous le linge. Ça sent le lait ! Tu sens, Nina ? Oui. Le linge blanc a de petits trous. Le carrelage est froid sous les chaussures. On reste près du marbre. Le marbre du comptoir est lisse. Le linge sent le lait, un peu. Nina regarde par un trou du linge. Je vois le morceau. Par un trou, Nina ? Oui, maman. Je le veux, maintenant. En ce moment, Nina serre la veste. Le sol est froid sous ses chaussures. Une feuille craque sous un morceau. Celui-là ! Nina se dresse sur les pointes. Un petit morceau beige attend sous le verre. Nina tend la main trop vite. Je le prends ! Le doigt tape le verre. Oh. Le morceau reste sous la cloche. La dame ne lève pas les yeux. Le sourire de Nina disparaît. Il ne vient pas. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Le fromage est sous le verre. Tu le vois, Nina ? Les épaules de Nina tombent un peu. Ça serre, dans son ventre. L'éclat de cloche tremble, puis tient. Papa se baisse à sa hauteur. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>éclat de cloche</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,43 +1324,66 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_fromage_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un linge blanc a de petits trous.
-narrateur|Un rayon y passe, tout pâle.
-narrateur|Ça sent le lait froid.
-narrateur|Des fromages ronds dorment dessous.
-narrateur|Une cloche de verre tient un morceau.
-narrateur|Le verre est un peu embué, tout doux.
-papa|Tu as vu les trous, Nina ?
-enfant-f|Comme des fenêtres.
-maman|Tout petits.
-narrateur|Papa pousse la porte tout doux.
+          <t>narrateur|Le verre de la cloche est froid.
+narrateur|Un rayon pâle y glisse.
+narrateur|Sur le verre, un éclat de cloche luit.
+enfant-f|Il brille, papa.
+papa|Tu le vois, sur le verre ?
+narrateur|Nina pose un doigt, un instant.
+narrateur|Le verre pique un peu le doigt.
+enfant-f|Il est froid.
+maman|La veste, un bouton de plus.
+papa|Voilà.
 narrateur|Un souffle frais sort de la boutique.
-narrateur|Une petite cloche fait ding, tout bas.
-maman|Tu as senti le lait, Nina ?
+enfant-f|J'ai les joues froides.
+papa|On avance.
+maman|Tu restes près de nous ?
 enfant-f|Oui, maman.
-enfant-f|C'est frais.
-papa|Comme le matin.
+narrateur|Ça sent le lait, près du verre.
+narrateur|Des ronds dorment sous le linge.
+enfant-f|Ça sent le lait !
+maman|Tu sens, Nina ?
+enfant-f|Oui.
+narrateur|Le linge blanc a de petits trous.
 narrateur|Le carrelage est froid sous les chaussures.
-maman|Tu as les pieds froids, Nina ?
-enfant-f|Un peu, maman.
-narrateur|En ce moment, Nina s'arrête au comptoir.
-narrateur|Un petit morceau beige est sur une feuille.
-narrateur|La feuille craque un peu.
-enfant-f|Celui-là, papa.
-papa|On s'approche du comptoir.
-maman|Elle plie encore le linge.
-narrateur|Nina se tient près de maman.
-narrateur|Elle regarde par un trou du linge.
+papa|On reste près du marbre.
+narrateur|Le marbre du comptoir est lisse.
+narrateur|Le linge sent le lait, un peu.
+narrateur|Nina regarde par un trou du linge.
 enfant-f|Je vois le morceau.
-maman|Oui.
-narrateur|La dame pose le linge.
-narrateur|Elle lève les yeux.
-papa|Tu demandes, Nina.</t>
+maman|Par un trou, Nina ?
+enfant-f|Oui, maman.
+enfant-f|Je le veux, maintenant.
+narrateur|En ce moment, Nina serre la veste.
+narrateur|Le sol est froid sous ses chaussures.
+narrateur|Une feuille craque sous un morceau.
+enfant-f|Celui-là !
+narrateur|Nina se dresse sur les pointes.
+narrateur|Un petit morceau beige attend sous le verre.
+narrateur|Nina tend la main trop vite.
+enfant-f|Je le prends !
+narrateur|Le doigt tape le verre.
+enfant-f|Oh.
+narrateur|Le morceau reste sous la cloche.
+narrateur|La dame ne lève pas les yeux.
+narrateur|Le sourire de Nina disparaît.
+enfant-f|Il ne vient pas.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+maman|Le fromage est sous le verre.
+papa|Tu le vois, Nina ?
+narrateur|Les épaules de Nina tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|L'éclat de cloche tremble, puis tient.
+narrateur|Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1392,17 +1415,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Nina veut le morceau. Que dit-elle ?</t>
+          <t>Nina parle à la dame. Que dit-elle ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nina veut le morceau. Que dit-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina parle à la &lt;emphasis level="moderate"&gt;dame&lt;/emphasis&gt;. Que dit-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;David parle à la dame. Que dit-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nina parle à la &lt;emphasis&gt;dame&lt;/emphasis&gt;. Que dit-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1412,7 +1435,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>bonjour | s'il te plaît | merci | bonjour merci</t>
+          <t>bonjour | s'il te plaît | merci | bonjour merci | s'il vous plaît</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1465,7 +1488,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1473,10 +1496,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1491,34 +1514,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>dame</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1527,13 +1554,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1543,12 +1570,12 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_parle_a_la_dame_avec_bonjour; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Nina veut le morceau.
+          <t>narrateur|Nina parle à la dame.
 narrateur|Que dit-elle ?</t>
         </is>
       </c>
@@ -1576,17 +1603,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Un morceau, s'il te plaît. Celui de la feuille. La dame glisse le morceau dans un sac. Le sac est frais, un peu lourd. Merci. Merci. Nina tient le sac contre son manteau. Ça sent le lait, tout près. Il est froid, papa. Oui. Comme le carrelage. Mes mains sont froides. On les met dans tes poches ? Le sac aussi. Tout contre toi. Le linge blanc couvre encore les ronds. Le rayon pâle n'y passe plus. On rentre ? Oui, papa.</t>
+          <t>Nina avance trop vite vers le verre. Celui-là, maintenant ! Sa voix se mélange près du linge. Oh. Le morceau reste sous la cloche. Nina refuse de foncer, cette fois. Nina referme la main. Elle écoute le verre, un instant. Tu veux venir près du marbre ? Papa s'accroupit à la même hauteur. Nina pose un pied sur le carrelage. Bonjour. Celui-là. S'il te plaît. Derrière le verre, une main se tend. La dame glisse le morceau dans un sac. Le papier enveloppe le fromage. Le sac est froid contre la veste. Merci. Merci, Nina. Papa a entendu toute la phrase. Le ventre de Nina se desserre. Les épaules se relèvent un peu. Tu as les mains au froid ? Un peu, maman. Ça sent le lait, tout près. Le fromage est à moi. Il est dans tes mains. Nina pose une main sur le sac. Le papier est un peu rêche. Le verre de la cloche se tait.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Un morceau, s'il te plaît. Celui de la feuille. La dame glisse le morceau dans un sac. Le sac est frais, un peu lourd. Merci. Merci. Nina tient le sac contre son manteau. Ça sent le lait, tout près. Il est froid, papa. Oui. Comme le carrelage. Mes mains sont froides. On les met dans tes poches ? Le sac aussi. Tout contre toi. Le linge blanc couvre encore les ronds. Le rayon pâle n'y passe plus. On rentre ? Oui, papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina avance trop vite vers le verre. Celui-là, maintenant ! Sa voix se mélange près du linge. Oh. Le morceau reste sous la cloche. Nina refuse de foncer, cette fois. Nina referme la main. Elle écoute le verre, un instant. Tu veux venir près du marbre ? Papa s'accroupit à la même hauteur. Nina pose un pied sur le carrelage. &lt;emphasis level="moderate"&gt;Bonjour&lt;/emphasis&gt;. Celui-là. S'il te plaît. Derrière le verre, une main se tend. La dame glisse le morceau dans un sac. Le papier enveloppe le fromage. Le sac est froid contre la veste. Merci. Merci, Nina. Papa a entendu toute la phrase. Le ventre de Nina se desserre. Les épaules se relèvent un peu. Tu as les mains au froid ? Un peu, maman. Ça sent le lait, tout près. Le fromage est à moi. Il est dans tes mains. Nina pose une main sur le sac. Le papier est un peu rêche. Le verre de la cloche se tait.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;David a dit &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Il a dit s'il te plaît. Il a dit merci. Papa et maman ont entendu.&lt;/slow&gt; [pause]</t>
+          <t>Nina avance trop vite vers le verre. Celui-là, maintenant ! Sa voix se mélange près du linge. Oh. Le morceau reste sous la cloche. Nina refuse de foncer, cette fois. Nina referme la main. Elle écoute le verre, un instant. Tu veux venir près du marbre ? Papa s'accroupit à la même hauteur. Nina pose un pied sur le carrelage. &lt;emphasis&gt;Bonjour&lt;/emphasis&gt;. Celui-là. S'il te plaît. Derrière le verre, une main se tend. La dame glisse le morceau dans un sac. Le papier enveloppe le fromage. Le sac est froid contre la veste. Merci. Merci, Nina. Papa a entendu toute la phrase. Le ventre de Nina se desserre. Les épaules se relèvent un peu. Tu as les mains au froid ? Un peu, maman. Ça sent le lait, tout près. Le fromage est à moi. Il est dans tes mains. Nina pose une main sur le sac. Le papier est un peu rêche. Le verre de la cloche se tait. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1633,18 +1660,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1667,30 +1694,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>Bonjour</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1699,10 +1726,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1711,36 +1738,46 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=bonjour_s_il_te_plait_merci_vecus; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-f|Bonjour.
-maman|Bonjour.
-enfant-f|Un morceau, s'il te plaît.
-enfant-f|Celui de la feuille.
+          <t>narrateur|Nina avance trop vite vers le verre.
+enfant-f|Celui-là, maintenant !
+narrateur|Sa voix se mélange près du linge.
+enfant-f|Oh.
+narrateur|Le morceau reste sous la cloche.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Nina referme la main.
+narrateur|Elle écoute le verre, un instant.
+papa|Tu veux venir près du marbre ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Nina pose un pied sur le carrelage.
+enfant-f|Bonjour.
+enfant-f|Celui-là.
+enfant-f|S'il te plaît.
+narrateur|Derrière le verre, une main se tend.
 narrateur|La dame glisse le morceau dans un sac.
-narrateur|Le sac est frais, un peu lourd.
+narrateur|Le papier enveloppe le fromage.
+narrateur|Le sac est froid contre la veste.
 enfant-f|Merci.
-papa|Merci.
-narrateur|Nina tient le sac contre son manteau.
+papa|Merci, Nina.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Nina se desserre.
+narrateur|Les épaules se relèvent un peu.
+maman|Tu as les mains au froid ?
+enfant-f|Un peu, maman.
 narrateur|Ça sent le lait, tout près.
-enfant-f|Il est froid, papa.
-papa|Oui.
-maman|Comme le carrelage.
-enfant-f|Mes mains sont froides.
-papa|On les met dans tes poches ?
-enfant-f|Le sac aussi.
-maman|Tout contre toi.
-narrateur|Le linge blanc couvre encore les ronds.
-narrateur|Le rayon pâle n'y passe plus.
-papa|On rentre ?
-enfant-f|Oui, papa.</t>
+enfant-f|Le fromage est à moi.
+maman|Il est dans tes mains.
+narrateur|Nina pose une main sur le sac.
+narrateur|Le papier est un peu rêche.
+narrateur|Le verre de la cloche se tait.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1772,17 +1809,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent par la rue étroite. Les pavés sont secs, maintenant. Nina tient encore le bord du sac. À la maison, papa ouvre le sac. Le morceau est pâle, un peu doux au nez. Tu veux sentir ? Oui, maman. S'il te plaît. Nina se penche. Ça sent le lait. On le met sur le pain ? Oui. Papa pose un petit carré sur une tartine. Merci, papa. Merci, Nina. Le sac reste frais, sur la table. Tes mains sont moins froides ? Un peu. Le pain est doux. Nina croque un tout petit bout. C'est frais. Oui.</t>
+          <t>Nina veut soulever la cloche, d'un coup. Je le sens, tout près ! Elle prend le verre trop vite. La cloche glisse sur le marbre. Oh. Nina avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Nina observe le verre, écoute la boutique. Sur le verre, un éclat de cloche luit. Là, près de la cloche. Nina pose la cloche, sans se presser. Le verre fait un petit toc. Elle reste là. Tu le vois, toi ? Oui, sur le verre. Nina tient le sac des deux mains. Le papier est rêche, un peu froid. Il est froid, papa. Tu le portes jusqu'à la porte ? Oui, papa. On sort ? Oui, maman. La porte s'ouvre. L'air frais revient sur les joues. Nina serre le sac contre elle. Il reste froid. On marche. Le sac penche, puis se cale. Je le tiens. On avance. Nina passe le seuil de pierre. La pierre est froide, un peu.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent par la rue étroite. Les pavés sont secs, maintenant. Nina tient encore le bord du sac. À la maison, papa ouvre le sac. Le morceau est pâle, un peu doux au nez. Tu veux sentir ? Oui, maman. S'il te plaît. Nina se penche. Ça sent le lait. On le met sur le pain ? Oui. Papa pose un petit carré sur une tartine. Merci, papa. Merci, Nina. Le sac reste frais, sur la table. Tes mains sont moins froides ? Un peu. Le pain est doux. Nina croque un tout petit bout. C'est frais. Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina veut soulever la &lt;emphasis level="moderate"&gt;cloche&lt;/emphasis&gt;, d'un coup. Je le sens, tout près ! Elle prend le verre trop vite. La cloche glisse sur le marbre. Oh. Nina avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Nina observe le verre, écoute la boutique. Sur le verre, un éclat de cloche luit. Là, près de la cloche. Nina pose la cloche, sans se presser. Le verre fait un petit toc. Elle reste là. Tu le vois, toi ? Oui, sur le verre. Nina tient le sac des deux mains. Le papier est rêche, un peu froid. Il est froid, papa. Tu le portes jusqu'à la porte ? Oui, papa. On sort ? Oui, maman. La porte s'ouvre. L'air frais revient sur les joues. Nina serre le sac contre elle. Il reste froid. On marche. Le sac penche, puis se cale. Je le tiens. On avance. Nina passe le seuil de pierre. La pierre est froide, un peu.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;David sent le fromage. Papa range le sac.&lt;/slow&gt; [pause]</t>
+          <t>Nina veut soulever la &lt;emphasis&gt;cloche&lt;/emphasis&gt;, d'un coup. Je le sens, tout près ! Elle prend le verre trop vite. La cloche glisse sur le marbre. Oh. Nina avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Nina observe le verre, écoute la boutique. Sur le verre, un éclat de cloche luit. Là, près de la cloche. Nina pose la cloche, sans se presser. Le verre fait un petit toc. Elle reste là. Tu le vois, toi ? Oui, sur le verre. Nina tient le sac des deux mains. Le papier est rêche, un peu froid. Il est froid, papa. Tu le portes jusqu'à la porte ? Oui, papa. On sort ? Oui, maman. La porte s'ouvre. L'air frais revient sur les joues. Nina serre le sac contre elle. Il reste froid. On marche. Le sac penche, puis se cale. Je le tiens. On avance. Nina passe le seuil de pierre. La pierre est froide, un peu. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1829,18 +1866,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1861,28 +1898,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>cloche</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1891,10 +1932,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1903,38 +1944,54 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_sur_la_cloche; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Ils rentrent par la rue étroite.
-narrateur|Les pavés sont secs, maintenant.
-narrateur|Nina tient encore le bord du sac.
-narrateur|À la maison, papa ouvre le sac.
-narrateur|Le morceau est pâle, un peu doux au nez.
-maman|Tu veux sentir ?
+          <t>narrateur|Nina veut soulever la cloche, d'un coup.
+enfant-f|Je le sens, tout près !
+narrateur|Elle prend le verre trop vite.
+narrateur|La cloche glisse sur le marbre.
+enfant-f|Oh.
+narrateur|Nina avance les mains.
+narrateur|Puis elle s'arrête net.
+enfant-f|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Nina observe le verre, écoute la boutique.
+narrateur|Sur le verre, un éclat de cloche luit.
+enfant-f|Là, près de la cloche.
+narrateur|Nina pose la cloche, sans se presser.
+narrateur|Le verre fait un petit toc.
+enfant-f|Elle reste là.
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur le verre.
+narrateur|Nina tient le sac des deux mains.
+narrateur|Le papier est rêche, un peu froid.
+enfant-f|Il est froid, papa.
+papa|Tu le portes jusqu'à la porte ?
+enfant-f|Oui, papa.
+maman|On sort ?
 enfant-f|Oui, maman.
-enfant-f|S'il te plaît.
-narrateur|Nina se penche.
-enfant-f|Ça sent le lait.
-maman|On le met sur le pain ?
-enfant-f|Oui.
-narrateur|Papa pose un petit carré sur une tartine.
-enfant-f|Merci, papa.
-papa|Merci, Nina.
-narrateur|Le sac reste frais, sur la table.
-maman|Tes mains sont moins froides ?
-enfant-f|Un peu.
-papa|Le pain est doux.
-narrateur|Nina croque un tout petit bout.
-enfant-f|C'est frais.
-maman|Oui.</t>
+narrateur|La porte s'ouvre.
+narrateur|L'air frais revient sur les joues.
+narrateur|Nina serre le sac contre elle.
+enfant-f|Il reste froid.
+papa|On marche.
+narrateur|Le sac penche, puis se cale.
+enfant-f|Je le tiens.
+maman|On avance.
+narrateur|Nina passe le seuil de pierre.
+narrateur|La pierre est froide, un peu.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>pain</t>
+          <t>papier,porte</t>
         </is>
       </c>
     </row>
@@ -1961,17 +2018,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le sac frais repose près du pain. Il reste un bout, tout pâle. Bonne journée, Nina. Il sentait le lait, ton morceau.</t>
+          <t>Le verre brillait, papa. Tu le vois, comme dans la boutique ? Oui, sur la cloche. Nina pose le sac contre la veste. On le garde au froid ? Oui, maman. Le lait sentait bon. Il est contre toi. Un souffle froid monte du papier. Nina respire, plus large. On rentre ? Oui. Les joues de Nina se réchauffent. Le sac reste froid sous la main. Un éclat de cloche reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le sac frais repose près du pain. Il reste un bout, tout pâle. Bonne journée, Nina. Il sentait le lait, ton morceau.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le verre brillait, papa. Tu le vois, comme dans la boutique ? Oui, sur la cloche. Nina pose le sac contre la veste. On le garde au froid ? Oui, maman. Le lait sentait bon. Il est contre toi. Un souffle froid monte du papier. Nina respire, plus large. On rentre ? Oui. Les joues de Nina se réchauffent. Le sac reste froid sous la main. Un &lt;emphasis level="moderate"&gt;éclat de cloche&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le verre brillait, papa. Tu le vois, comme dans la boutique ? Oui, sur la cloche. Nina pose le sac contre la veste. On le garde au froid ? Oui, maman. Le lait sentait bon. Il est contre toi. Un souffle froid monte du papier. Nina respire, plus large. On rentre ? Oui. Les joues de Nina se réchauffent. Le sac reste froid sous la main. Un &lt;emphasis&gt;éclat de cloche&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2018,7 +2075,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2026,10 +2083,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2038,12 +2095,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2052,17 +2109,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cloche</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2071,11 +2132,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2084,27 +2145,47 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le sac frais repose près du pain.
-narrateur|Il reste un bout, tout pâle.
-maman|Bonne journée, Nina.
-papa|Il sentait le lait, ton morceau.</t>
+          <t>enfant-f|Le verre brillait, papa.
+papa|Tu le vois, comme dans la boutique ?
+enfant-f|Oui, sur la cloche.
+narrateur|Nina pose le sac contre la veste.
+maman|On le garde au froid ?
+enfant-f|Oui, maman.
+enfant-f|Le lait sentait bon.
+maman|Il est contre toi.
+narrateur|Un souffle froid monte du papier.
+narrateur|Nina respire, plus large.
+papa|On rentre ?
+enfant-f|Oui.
+narrateur|Les joues de Nina se réchauffent.
+narrateur|Le sac reste froid sous la main.
+narrateur|Un éclat de cloche reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>cloche</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2217,6 +2298,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>